<commit_message>
Updated Manual chart builder, Chart type change, Kpi cards alignment
</commit_message>
<xml_diff>
--- a/user file log.xlsx
+++ b/user file log.xlsx
@@ -1147,7 +1147,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F22"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1489,9 +1489,109 @@
         <v>no join configs</v>
       </c>
     </row>
+    <row r="18">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" t="str">
+        <v>sales_dataset_100_rows_multi_year.csv</v>
+      </c>
+      <c r="C18" t="str">
+        <v>3/19/2026</v>
+      </c>
+      <c r="D18" t="str">
+        <v>12:10:38 AM</v>
+      </c>
+      <c r="E18" t="str">
+        <v>OrderID, Region, Category, Product, Sales, Quantity, Profit, OrderDate</v>
+      </c>
+      <c r="F18" t="str">
+        <v>no join configs</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" t="str">
+        <v>sales_dataset_100_rows_multi_year.csv</v>
+      </c>
+      <c r="C19" t="str">
+        <v>3/19/2026</v>
+      </c>
+      <c r="D19" t="str">
+        <v>11:14:05 PM</v>
+      </c>
+      <c r="E19" t="str">
+        <v>OrderID, OrderDate, Region, Category, Product, Sales, Quantity, Profit</v>
+      </c>
+      <c r="F19" t="str">
+        <v>no join configs</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" t="str">
+        <v>sales_dataset_100_rows_multi_year.csv</v>
+      </c>
+      <c r="C20" t="str">
+        <v>3/20/2026</v>
+      </c>
+      <c r="D20" t="str">
+        <v>12:03:16 AM</v>
+      </c>
+      <c r="E20" t="str">
+        <v>OrderID, OrderDate, Region, Category, Product, Sales, Quantity, Profit</v>
+      </c>
+      <c r="F20" t="str">
+        <v>no join configs</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21" t="str">
+        <v>sales_dataset_100_rows_multi_year.csv</v>
+      </c>
+      <c r="C21" t="str">
+        <v>3/20/2026</v>
+      </c>
+      <c r="D21" t="str">
+        <v>6:59:30 PM</v>
+      </c>
+      <c r="E21" t="str">
+        <v>OrderID, OrderDate, Region, Category, Product, Sales, Quantity, Profit</v>
+      </c>
+      <c r="F21" t="str">
+        <v>no join configs</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22" t="str">
+        <v>sales_dataset_100_rows_multi_year.csv</v>
+      </c>
+      <c r="C22" t="str">
+        <v>3/23/2026</v>
+      </c>
+      <c r="D22" t="str">
+        <v>6:36:40 PM</v>
+      </c>
+      <c r="E22" t="str">
+        <v>OrderID, OrderDate, Region, Category, Product, Sales, Quantity, Profit</v>
+      </c>
+      <c r="F22" t="str">
+        <v>no join configs</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F17"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F22"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>